<commit_message>
#16 Battery Peripheral Link update in Client BOM
</commit_message>
<xml_diff>
--- a/Design-Files/Pukk-Display-Module-v1.0/BOM/Client-BOM-Pukk-Display-Module-v1.0.xlsx
+++ b/Design-Files/Pukk-Display-Module-v1.0/BOM/Client-BOM-Pukk-Display-Module-v1.0.xlsx
@@ -970,12 +970,6 @@
     <t>Battery Cell</t>
   </si>
   <si>
-    <t>LR621</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> AG1 LR621 364 V364 164 531 SR621 SR621SW SR60 CX60 1.55V Alkaline Battery For Watch Car Key Remote Toy Button Coin Cell</t>
-  </si>
-  <si>
     <t>Alibaba</t>
   </si>
   <si>
@@ -986,6 +980,12 @@
   </si>
   <si>
     <t>KD050FHFID103</t>
+  </si>
+  <si>
+    <t>MC621 621 Button lithium Industrial Lithium Battery</t>
+  </si>
+  <si>
+    <t>MC621</t>
   </si>
 </sst>
 </file>
@@ -1222,9 +1222,6 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1239,6 +1236,9 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="6" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1553,10 +1553,10 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
-      <c r="L1" s="14"/>
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19"/>
+      <c r="L1" s="19"/>
     </row>
     <row r="2" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -3121,29 +3121,29 @@
       <c r="C49" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="D49" s="15" t="s">
+      <c r="D49" s="14" t="s">
         <v>73</v>
       </c>
-      <c r="E49" s="16" t="s">
+      <c r="E49" s="15" t="s">
         <v>133</v>
       </c>
-      <c r="F49" s="15" t="s">
+      <c r="F49" s="14" t="s">
         <v>179</v>
       </c>
-      <c r="G49" s="16" t="s">
+      <c r="G49" s="15" t="s">
         <v>225</v>
       </c>
-      <c r="H49" s="15" t="s">
+      <c r="H49" s="14" t="s">
         <v>249</v>
       </c>
-      <c r="I49" s="16" t="s">
+      <c r="I49" s="15" t="s">
         <v>291</v>
       </c>
-      <c r="J49" s="15">
-        <v>1</v>
-      </c>
-      <c r="K49" s="15"/>
-      <c r="L49" s="17" t="s">
+      <c r="J49" s="14">
+        <v>1</v>
+      </c>
+      <c r="K49" s="14"/>
+      <c r="L49" s="16" t="s">
         <v>302</v>
       </c>
     </row>
@@ -3222,29 +3222,29 @@
       <c r="C52" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="D52" s="15" t="s">
+      <c r="D52" s="14" t="s">
         <v>76</v>
       </c>
-      <c r="E52" s="16" t="s">
+      <c r="E52" s="15" t="s">
         <v>137</v>
       </c>
-      <c r="F52" s="15" t="s">
+      <c r="F52" s="14" t="s">
         <v>178</v>
       </c>
-      <c r="G52" s="16" t="s">
+      <c r="G52" s="15" t="s">
         <v>229</v>
       </c>
-      <c r="H52" s="15" t="s">
+      <c r="H52" s="14" t="s">
         <v>249</v>
       </c>
-      <c r="I52" s="16" t="s">
+      <c r="I52" s="15" t="s">
         <v>291</v>
       </c>
-      <c r="J52" s="15">
+      <c r="J52" s="14">
         <v>2</v>
       </c>
-      <c r="K52" s="15"/>
-      <c r="L52" s="17" t="s">
+      <c r="K52" s="14"/>
+      <c r="L52" s="16" t="s">
         <v>302</v>
       </c>
     </row>
@@ -3772,10 +3772,10 @@
       <c r="J68" s="7">
         <v>1</v>
       </c>
-      <c r="K68" s="19" t="s">
+      <c r="K68" s="18" t="s">
         <v>311</v>
       </c>
-      <c r="L68" s="18" t="s">
+      <c r="L68" s="17" t="s">
         <v>309</v>
       </c>
     </row>
@@ -3808,12 +3808,12 @@
       <c r="J69" s="7">
         <v>1</v>
       </c>
-      <c r="K69" s="19" t="s">
+      <c r="K69" s="18" t="s">
         <v>311</v>
       </c>
-      <c r="L69" s="18"/>
-    </row>
-    <row r="70" spans="1:12" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L69" s="17"/>
+    </row>
+    <row r="70" spans="1:12" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B70" s="11">
         <f t="shared" si="1"/>
         <v>68</v>
@@ -3825,13 +3825,13 @@
         <v>315</v>
       </c>
       <c r="E70" s="8" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="F70" s="7" t="s">
         <v>303</v>
       </c>
       <c r="G70" s="8" t="s">
-        <v>316</v>
+        <v>321</v>
       </c>
       <c r="H70" s="7" t="s">
         <v>301</v>
@@ -3842,10 +3842,10 @@
       <c r="J70" s="7">
         <v>1</v>
       </c>
-      <c r="K70" s="19" t="s">
+      <c r="K70" s="18" t="s">
         <v>311</v>
       </c>
-      <c r="L70" s="18"/>
+      <c r="L70" s="17"/>
     </row>
     <row r="71" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B71" s="11">
@@ -3856,16 +3856,16 @@
         <v>304</v>
       </c>
       <c r="D71" s="7" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="E71" s="8" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="F71" s="7" t="s">
         <v>303</v>
       </c>
       <c r="G71" s="8" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="H71" s="7" t="s">
         <v>301</v>
@@ -3876,10 +3876,10 @@
       <c r="J71" s="7">
         <v>1</v>
       </c>
-      <c r="K71" s="19" t="s">
-        <v>318</v>
-      </c>
-      <c r="L71" s="18"/>
+      <c r="K71" s="18" t="s">
+        <v>316</v>
+      </c>
+      <c r="L71" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -3888,8 +3888,8 @@
   <hyperlinks>
     <hyperlink ref="K68" r:id="rId1"/>
     <hyperlink ref="K69" r:id="rId2"/>
-    <hyperlink ref="K70" r:id="rId3"/>
-    <hyperlink ref="K71" r:id="rId4"/>
+    <hyperlink ref="K71" r:id="rId3"/>
+    <hyperlink ref="K70" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId5"/>

</xml_diff>

<commit_message>
#18 Schematic and PCB with deliverables Completed.
</commit_message>
<xml_diff>
--- a/Design-Files/Pukk-Display-Module-v1.0/BOM/Client-BOM-Pukk-Display-Module-v1.0.xlsx
+++ b/Design-Files/Pukk-Display-Module-v1.0/BOM/Client-BOM-Pukk-Display-Module-v1.0.xlsx
@@ -750,9 +750,6 @@
     <t>ST1L05APU33R</t>
   </si>
   <si>
-    <t>DF40C-30DP-0.4V(51)</t>
-  </si>
-  <si>
     <t>SN74HC14QDRQ1</t>
   </si>
   <si>
@@ -986,6 +983,9 @@
   </si>
   <si>
     <t>MC621</t>
+  </si>
+  <si>
+    <t>DF40C-100DS-0.4V(51)</t>
   </si>
 </sst>
 </file>
@@ -1579,19 +1579,19 @@
         <v>190</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="J2" s="5" t="s">
+        <v>297</v>
+      </c>
+      <c r="K2" s="5" t="s">
+        <v>309</v>
+      </c>
+      <c r="L2" s="5" t="s">
         <v>298</v>
-      </c>
-      <c r="K2" s="5" t="s">
-        <v>310</v>
-      </c>
-      <c r="L2" s="5" t="s">
-        <v>299</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1616,10 +1616,10 @@
         <v>157</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="J3" s="7">
         <v>1</v>
@@ -1649,10 +1649,10 @@
         <v>191</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="J4" s="9">
         <v>2</v>
@@ -1682,10 +1682,10 @@
         <v>192</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="J5" s="7">
         <v>1</v>
@@ -1715,10 +1715,10 @@
         <v>193</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="J6" s="9">
         <v>1</v>
@@ -1748,10 +1748,10 @@
         <v>194</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="J7" s="7">
         <v>1</v>
@@ -1781,10 +1781,10 @@
         <v>195</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="J8" s="9">
         <v>7</v>
@@ -1814,10 +1814,10 @@
         <v>196</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="J9" s="7">
         <v>1</v>
@@ -1847,10 +1847,10 @@
         <v>197</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="J10" s="9">
         <v>3</v>
@@ -1880,10 +1880,10 @@
         <v>198</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="J11" s="7">
         <v>2</v>
@@ -1913,10 +1913,10 @@
         <v>199</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="J12" s="9">
         <v>5</v>
@@ -1946,10 +1946,10 @@
         <v>200</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="J13" s="7">
         <v>2</v>
@@ -1979,10 +1979,10 @@
         <v>201</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="J14" s="9">
         <v>1</v>
@@ -2012,10 +2012,10 @@
         <v>202</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I15" s="8" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="J15" s="7">
         <v>1</v>
@@ -2045,10 +2045,10 @@
         <v>203</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="J16" s="9">
         <v>3</v>
@@ -2072,16 +2072,16 @@
         <v>107</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="G17" s="8" t="s">
         <v>204</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="I17" s="8" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="J17" s="7">
         <v>1</v>
@@ -2111,10 +2111,10 @@
         <v>205</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="J18" s="9">
         <v>1</v>
@@ -2144,10 +2144,10 @@
         <v>206</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I19" s="8" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="J19" s="7">
         <v>2</v>
@@ -2177,10 +2177,10 @@
         <v>207</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="J20" s="9">
         <v>1</v>
@@ -2210,10 +2210,10 @@
         <v>208</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="I21" s="10" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="J21" s="7">
         <v>1</v>
@@ -2243,10 +2243,10 @@
         <v>209</v>
       </c>
       <c r="H22" s="9" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="I22" s="10" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="J22" s="9">
         <v>1</v>
@@ -2276,10 +2276,10 @@
         <v>210</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="I23" s="10" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="J23" s="7">
         <v>1</v>
@@ -2309,10 +2309,10 @@
         <v>211</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="I24" s="10" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="J24" s="9">
         <v>10</v>
@@ -2342,10 +2342,10 @@
         <v>212</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="I25" s="10" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="J25" s="7">
         <v>3</v>
@@ -2375,10 +2375,10 @@
         <v>213</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="I26" s="10" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="J26" s="9">
         <v>3</v>
@@ -2408,10 +2408,10 @@
         <v>214</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="I27" s="10" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="J27" s="7">
         <v>1</v>
@@ -2441,10 +2441,10 @@
         <v>215</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="I28" s="10" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="J28" s="9">
         <v>1</v>
@@ -2474,10 +2474,10 @@
         <v>216</v>
       </c>
       <c r="H29" s="7" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="I29" s="10" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="J29" s="7">
         <v>1</v>
@@ -2507,10 +2507,10 @@
         <v>217</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="I30" s="10" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="J30" s="9">
         <v>1</v>
@@ -2534,16 +2534,16 @@
         <v>121</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="G31" s="8" t="s">
         <v>171</v>
       </c>
       <c r="H31" s="7" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="I31" s="10" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="J31" s="7">
         <v>1</v>
@@ -2567,16 +2567,16 @@
         <v>122</v>
       </c>
       <c r="F32" s="7" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="G32" s="10" t="s">
         <v>172</v>
       </c>
       <c r="H32" s="9" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="I32" s="10" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="J32" s="9">
         <v>1</v>
@@ -2600,16 +2600,16 @@
         <v>123</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="G33" s="8" t="s">
         <v>173</v>
       </c>
       <c r="H33" s="7" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="I33" s="10" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="J33" s="7">
         <v>1</v>
@@ -2633,16 +2633,16 @@
         <v>124</v>
       </c>
       <c r="F34" s="7" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="G34" s="10" t="s">
         <v>174</v>
       </c>
       <c r="H34" s="9" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="I34" s="10" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="J34" s="9">
         <v>1</v>
@@ -2672,10 +2672,10 @@
         <v>218</v>
       </c>
       <c r="H35" s="7" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="I35" s="10" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="J35" s="7">
         <v>1</v>
@@ -2699,16 +2699,16 @@
         <v>126</v>
       </c>
       <c r="F36" s="7" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="G36" s="10" t="s">
         <v>175</v>
       </c>
       <c r="H36" s="9" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="I36" s="10" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="J36" s="9">
         <v>1</v>
@@ -2738,10 +2738,10 @@
         <v>219</v>
       </c>
       <c r="H37" s="7" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="I37" s="8" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="J37" s="7">
         <v>1</v>
@@ -2771,10 +2771,10 @@
         <v>220</v>
       </c>
       <c r="H38" s="9" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="I38" s="10" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="J38" s="9">
         <v>2</v>
@@ -2804,10 +2804,10 @@
         <v>221</v>
       </c>
       <c r="H39" s="7" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="I39" s="10" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="J39" s="7">
         <v>1</v>
@@ -2837,10 +2837,10 @@
         <v>222</v>
       </c>
       <c r="H40" s="9" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="I40" s="10" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="J40" s="9">
         <v>1</v>
@@ -2870,10 +2870,10 @@
         <v>223</v>
       </c>
       <c r="H41" s="7" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="I41" s="10" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="J41" s="7">
         <v>2</v>
@@ -2903,10 +2903,10 @@
         <v>224</v>
       </c>
       <c r="H42" s="9" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I42" s="10" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="J42" s="9">
         <v>1</v>
@@ -2936,10 +2936,10 @@
         <v>225</v>
       </c>
       <c r="H43" s="7" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I43" s="8" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="J43" s="7">
         <v>1</v>
@@ -2969,10 +2969,10 @@
         <v>226</v>
       </c>
       <c r="H44" s="9" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I44" s="10" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="J44" s="9">
         <v>4</v>
@@ -3002,10 +3002,10 @@
         <v>227</v>
       </c>
       <c r="H45" s="7" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I45" s="8" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="J45" s="7">
         <v>1</v>
@@ -3035,10 +3035,10 @@
         <v>228</v>
       </c>
       <c r="H46" s="9" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I46" s="10" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="J46" s="9">
         <v>1</v>
@@ -3068,10 +3068,10 @@
         <v>229</v>
       </c>
       <c r="H47" s="7" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I47" s="8" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="J47" s="7">
         <v>12</v>
@@ -3101,10 +3101,10 @@
         <v>230</v>
       </c>
       <c r="H48" s="9" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I48" s="10" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="J48" s="9">
         <v>1</v>
@@ -3134,17 +3134,17 @@
         <v>225</v>
       </c>
       <c r="H49" s="14" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I49" s="15" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="J49" s="14">
         <v>1</v>
       </c>
       <c r="K49" s="14"/>
       <c r="L49" s="16" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="50" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3169,10 +3169,10 @@
         <v>231</v>
       </c>
       <c r="H50" s="9" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I50" s="10" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="J50" s="9">
         <v>2</v>
@@ -3202,10 +3202,10 @@
         <v>232</v>
       </c>
       <c r="H51" s="7" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I51" s="8" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="J51" s="7">
         <v>7</v>
@@ -3235,17 +3235,17 @@
         <v>229</v>
       </c>
       <c r="H52" s="14" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I52" s="15" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="J52" s="14">
         <v>2</v>
       </c>
       <c r="K52" s="14"/>
       <c r="L52" s="16" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="53" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3270,10 +3270,10 @@
         <v>233</v>
       </c>
       <c r="H53" s="7" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I53" s="8" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="J53" s="7">
         <v>1</v>
@@ -3303,10 +3303,10 @@
         <v>234</v>
       </c>
       <c r="H54" s="9" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I54" s="10" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="J54" s="9">
         <v>1</v>
@@ -3336,10 +3336,10 @@
         <v>235</v>
       </c>
       <c r="H55" s="7" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I55" s="8" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="J55" s="7">
         <v>5</v>
@@ -3369,10 +3369,10 @@
         <v>236</v>
       </c>
       <c r="H56" s="9" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I56" s="10" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="J56" s="9">
         <v>2</v>
@@ -3396,16 +3396,16 @@
         <v>145</v>
       </c>
       <c r="F57" s="7" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="G57" s="8" t="s">
         <v>182</v>
       </c>
       <c r="H57" s="7" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="I57" s="8" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="J57" s="7">
         <v>3</v>
@@ -3429,16 +3429,16 @@
         <v>146</v>
       </c>
       <c r="F58" s="7" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="G58" s="10" t="s">
         <v>183</v>
       </c>
       <c r="H58" s="9" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="I58" s="8" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="J58" s="9">
         <v>1</v>
@@ -3468,10 +3468,10 @@
         <v>237</v>
       </c>
       <c r="H59" s="7" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="I59" s="8" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="J59" s="7">
         <v>1</v>
@@ -3495,16 +3495,16 @@
         <v>148</v>
       </c>
       <c r="F60" s="7" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="G60" s="10" t="s">
         <v>238</v>
       </c>
       <c r="H60" s="9" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="I60" s="8" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="J60" s="9">
         <v>1</v>
@@ -3534,10 +3534,10 @@
         <v>239</v>
       </c>
       <c r="H61" s="7" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="I61" s="8" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="J61" s="7">
         <v>1</v>
@@ -3567,10 +3567,10 @@
         <v>240</v>
       </c>
       <c r="H62" s="9" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="I62" s="8" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="J62" s="9">
         <v>1</v>
@@ -3594,16 +3594,16 @@
         <v>151</v>
       </c>
       <c r="F63" s="7" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="G63" s="8" t="s">
         <v>186</v>
       </c>
       <c r="H63" s="7" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="I63" s="8" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="J63" s="7">
         <v>1</v>
@@ -3633,10 +3633,10 @@
         <v>241</v>
       </c>
       <c r="H64" s="9" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="I64" s="8" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="J64" s="9">
         <v>1</v>
@@ -3666,10 +3666,10 @@
         <v>242</v>
       </c>
       <c r="H65" s="7" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="I65" s="8" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="J65" s="7">
         <v>1</v>
@@ -3693,16 +3693,16 @@
         <v>154</v>
       </c>
       <c r="F66" s="7" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="G66" s="10" t="s">
-        <v>243</v>
+        <v>321</v>
       </c>
       <c r="H66" s="9" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="I66" s="8" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="J66" s="9">
         <v>2</v>
@@ -3729,13 +3729,13 @@
         <v>189</v>
       </c>
       <c r="G67" s="8" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="H67" s="7" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="I67" s="8" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="J67" s="7">
         <v>1</v>
@@ -3749,34 +3749,34 @@
         <v>66</v>
       </c>
       <c r="C68" s="12" t="s">
+        <v>303</v>
+      </c>
+      <c r="D68" s="7" t="s">
         <v>304</v>
       </c>
-      <c r="D68" s="7" t="s">
+      <c r="E68" s="8" t="s">
         <v>305</v>
       </c>
-      <c r="E68" s="8" t="s">
+      <c r="F68" s="7" t="s">
+        <v>302</v>
+      </c>
+      <c r="G68" s="8" t="s">
+        <v>307</v>
+      </c>
+      <c r="H68" s="7" t="s">
         <v>306</v>
       </c>
-      <c r="F68" s="7" t="s">
-        <v>303</v>
-      </c>
-      <c r="G68" s="8" t="s">
+      <c r="I68" s="8" t="s">
+        <v>300</v>
+      </c>
+      <c r="J68" s="7">
+        <v>1</v>
+      </c>
+      <c r="K68" s="18" t="s">
+        <v>310</v>
+      </c>
+      <c r="L68" s="17" t="s">
         <v>308</v>
-      </c>
-      <c r="H68" s="7" t="s">
-        <v>307</v>
-      </c>
-      <c r="I68" s="8" t="s">
-        <v>301</v>
-      </c>
-      <c r="J68" s="7">
-        <v>1</v>
-      </c>
-      <c r="K68" s="18" t="s">
-        <v>311</v>
-      </c>
-      <c r="L68" s="17" t="s">
-        <v>309</v>
       </c>
     </row>
     <row r="69" spans="1:12" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3785,31 +3785,31 @@
         <v>67</v>
       </c>
       <c r="C69" s="12" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D69" s="7" t="s">
+        <v>311</v>
+      </c>
+      <c r="E69" s="8" t="s">
         <v>312</v>
       </c>
-      <c r="E69" s="8" t="s">
+      <c r="F69" s="7" t="s">
+        <v>302</v>
+      </c>
+      <c r="G69" s="8" t="s">
+        <v>300</v>
+      </c>
+      <c r="H69" s="7" t="s">
         <v>313</v>
       </c>
-      <c r="F69" s="7" t="s">
-        <v>303</v>
-      </c>
-      <c r="G69" s="8" t="s">
-        <v>301</v>
-      </c>
-      <c r="H69" s="7" t="s">
-        <v>314</v>
-      </c>
       <c r="I69" s="8" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="J69" s="7">
         <v>1</v>
       </c>
       <c r="K69" s="18" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="L69" s="17"/>
     </row>
@@ -3819,31 +3819,31 @@
         <v>68</v>
       </c>
       <c r="C70" s="12" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D70" s="7" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="E70" s="8" t="s">
+        <v>319</v>
+      </c>
+      <c r="F70" s="7" t="s">
+        <v>302</v>
+      </c>
+      <c r="G70" s="8" t="s">
         <v>320</v>
       </c>
-      <c r="F70" s="7" t="s">
-        <v>303</v>
-      </c>
-      <c r="G70" s="8" t="s">
-        <v>321</v>
-      </c>
       <c r="H70" s="7" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="I70" s="8" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="J70" s="7">
         <v>1</v>
       </c>
       <c r="K70" s="18" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="L70" s="17"/>
     </row>
@@ -3853,31 +3853,31 @@
         <v>69</v>
       </c>
       <c r="C71" s="12" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D71" s="7" t="s">
+        <v>316</v>
+      </c>
+      <c r="E71" s="8" t="s">
         <v>317</v>
       </c>
-      <c r="E71" s="8" t="s">
+      <c r="F71" s="7" t="s">
+        <v>302</v>
+      </c>
+      <c r="G71" s="8" t="s">
         <v>318</v>
       </c>
-      <c r="F71" s="7" t="s">
-        <v>303</v>
-      </c>
-      <c r="G71" s="8" t="s">
-        <v>319</v>
-      </c>
       <c r="H71" s="7" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="I71" s="8" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="J71" s="7">
         <v>1</v>
       </c>
       <c r="K71" s="18" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="L71" s="17"/>
     </row>

</xml_diff>